<commit_message>
feat: import curriculum workbooks atomically
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,9 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R09d515f0c8f340b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="R9bfc6d7550ed4a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="3" r:id="R96baf1c322504db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Re224613c51564007"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="R91f89916cd924161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R4b0c6284a98d46cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Re106b35b58bb4c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R130678dc730e4b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="6" r:id="R5f6154b1c360498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,6 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -60,7 +66,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -88,6 +94,7 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -395,13 +402,14 @@
   <x:cols>
     <x:col min="1" max="1" width="9.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="5.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="8.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13.109999656677246" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -412,24 +420,27 @@
         <x:v>specialty_code</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
+        <x:v>curriculum_code</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
         <x:v>course</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="E1" s="6" t="str">
         <x:v>education_form</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="F1" s="6" t="str">
         <x:v>headcount</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>program_base</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>study_week_type</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>primary_building_code</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="J1" s="6" t="str">
         <x:v>subgroup_count</x:v>
       </x:c>
     </x:row>
@@ -440,25 +451,28 @@
       <x:c r="B2" s="7" t="str">
         <x:v>09.02.07</x:v>
       </x:c>
-      <x:c r="C2" s="7" t="n">
+      <x:c r="C2" s="7" t="str">
+        <x:v>UP-09.02.07-2026</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="str">
+      <x:c r="E2" s="7" t="str">
         <x:v>full_time</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="n">
+      <x:c r="F2" s="7" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="F2" s="7" t="str">
+      <x:c r="G2" s="7" t="str">
         <x:v>9_classes</x:v>
       </x:c>
-      <x:c r="G2" s="7" t="str">
+      <x:c r="H2" s="7" t="str">
         <x:v>six_days</x:v>
       </x:c>
-      <x:c r="H2" s="7" t="str">
+      <x:c r="I2" s="7" t="str">
         <x:v>MAIN</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="n">
+      <x:c r="J2" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -468,6 +482,196 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38.11000061035156" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34.11000061035156" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="5.110000133514404" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>specialty_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>specialty_name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>qualification</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>program_base</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>education_form</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>09.02.07</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Информационные системы и программирование</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Специалист по информационным системам</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>full_time</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="6.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.329999923706055" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>curriculum_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>specialty_code</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>admission_year</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>valid_from</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>valid_to</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>UP-09.02.07-2026</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>09.02.07</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F2" s="9"/>
+      <x:c r="G2" s="7" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.4399995803833" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>curriculum_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>discipline_code</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>discipline_name</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>section_code</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>semester</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>lesson_type</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>planned_hours</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>control_form</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>UP-09.02.07-2026</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>MDK.01.01</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Основы программирования</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>ПМ.01</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>practice</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>credit</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>

</xml_diff>

<commit_message>
feat: import student rosters atomically
Adds the Students worksheet to validation, preview, SQLite versioning, and activation. Rejects unnecessary personal-data columns and reports created, changed, and deactivated roster records before activation.
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Re224613c51564007"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="R91f89916cd924161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R4b0c6284a98d46cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Re106b35b58bb4c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R130678dc730e4b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="6" r:id="R5f6154b1c360498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R0b66a748ce064cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Ra4f0d0bf916245eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Rda476ef935e54673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Rba1499eab17b4a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R95051c2283c94fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="Rb38eaf2c31e54a31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="7" r:id="R8c0685a6fbaf441e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -675,6 +676,75 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>student_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>full_name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>group_code</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>enrollment_date</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>subgroup_codes</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>elective_codes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>S-001</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Петров Пётр Петрович</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>ИС-101</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F2" s="9"/>
+      <x:c r="G2" s="7" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>WEB</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="7.78000020980835" hidden="0" customWidth="1"/>

</xml_diff>

<commit_message>
feat: import room inventory atomically
Adds buildings, room types, equipment, and rooms to the canonical workbook, validation, versioned SQLite storage, CLI, API, and preview UI. Reports workload room shortages without discarding otherwise valid reference data.
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,13 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R0b66a748ce064cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Ra4f0d0bf916245eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Rda476ef935e54673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Rba1499eab17b4a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R95051c2283c94fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="Rb38eaf2c31e54a31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="7" r:id="R8c0685a6fbaf441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R6bd663c9ee7f46dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="R5144b9753eef4871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R0033eb10e51444f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Raa6879a5fa6047ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Rae5d6d3d1ce345ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R0e5f4c5af9ed4faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R145fb25f3ee6429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="Rbc87389d1d844a5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R68881d1edce44e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R429f29000edb401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="R2d4448ca7fc54ef6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -397,6 +401,198 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.110000133514404" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>room_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>room_name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>building_code</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>room_type_code</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>capacity</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>equipment_codes</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>MAIN-201</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Лаборатория 201</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>MAIN</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>COMPUTER_LAB</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>COMPUTERS</x:v>
+      </x:c>
+      <x:c r="G2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="5.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="9" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="21.559999465942383" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>workload_row_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>academic_year</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>semester</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>discipline_code</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>discipline_name</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>group_code</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>subgroup</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>stream</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>teacher_code</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
+        <x:v>lesson_type</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>total_academic_hours</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>event_duration_hours</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>recurrence</x:v>
+      </x:c>
+      <x:c r="N1" s="6" t="str">
+        <x:v>lesson_bundle_code</x:v>
+      </x:c>
+      <x:c r="O1" s="6" t="str">
+        <x:v>room_type</x:v>
+      </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>room_capacity</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>required_equipment_codes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>W-001</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>MDK.01.01</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>Основы программирования</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>ИС-101</x:v>
+      </x:c>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
+      <x:c r="I2" s="7" t="str">
+        <x:v>T-001</x:v>
+      </x:c>
+      <x:c r="J2" s="7" t="str">
+        <x:v>practice</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="L2" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M2" s="7" t="str">
+        <x:v>weekly</x:v>
+      </x:c>
+      <x:c r="N2" s="7"/>
+      <x:c r="O2" s="7" t="str">
+        <x:v>computer_lab</x:v>
+      </x:c>
+      <x:c r="P2" s="7" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="Q2" s="7" t="str">
+        <x:v>COMPUTERS</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -745,116 +941,103 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="7.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="5.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="17.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="17.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="9" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="16.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>workload_row_code</x:v>
+        <x:v>building_code</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>academic_year</x:v>
+        <x:v>building_name</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>semester</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>discipline_code</x:v>
-      </x:c>
-      <x:c r="E1" s="6" t="str">
-        <x:v>discipline_name</x:v>
-      </x:c>
-      <x:c r="F1" s="6" t="str">
-        <x:v>group_code</x:v>
-      </x:c>
-      <x:c r="G1" s="6" t="str">
-        <x:v>subgroup</x:v>
-      </x:c>
-      <x:c r="H1" s="6" t="str">
-        <x:v>stream</x:v>
-      </x:c>
-      <x:c r="I1" s="6" t="str">
-        <x:v>teacher_code</x:v>
-      </x:c>
-      <x:c r="J1" s="6" t="str">
-        <x:v>lesson_type</x:v>
-      </x:c>
-      <x:c r="K1" s="6" t="str">
-        <x:v>total_academic_hours</x:v>
-      </x:c>
-      <x:c r="L1" s="6" t="str">
-        <x:v>event_duration_hours</x:v>
-      </x:c>
-      <x:c r="M1" s="6" t="str">
-        <x:v>recurrence</x:v>
-      </x:c>
-      <x:c r="N1" s="6" t="str">
-        <x:v>lesson_bundle_code</x:v>
-      </x:c>
-      <x:c r="O1" s="6" t="str">
-        <x:v>room_type</x:v>
-      </x:c>
-      <x:c r="P1" s="6" t="str">
-        <x:v>room_capacity</x:v>
+        <x:v>active</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>W-001</x:v>
+        <x:v>MAIN</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026/2027</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="n">
+        <x:v>Главный корпус</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="str">
-        <x:v>MDK.01.01</x:v>
-      </x:c>
-      <x:c r="E2" s="7" t="str">
-        <x:v>Основы программирования</x:v>
-      </x:c>
-      <x:c r="F2" s="7" t="str">
-        <x:v>ИС-101</x:v>
-      </x:c>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-      <x:c r="I2" s="7" t="str">
-        <x:v>T-001</x:v>
-      </x:c>
-      <x:c r="J2" s="7" t="str">
-        <x:v>practice</x:v>
-      </x:c>
-      <x:c r="K2" s="7" t="n">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="L2" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="M2" s="7" t="str">
-        <x:v>weekly</x:v>
-      </x:c>
-      <x:c r="N2" s="7"/>
-      <x:c r="O2" s="7" t="str">
-        <x:v>computer_lab</x:v>
-      </x:c>
-      <x:c r="P2" s="7" t="n">
-        <x:v>25</x:v>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>room_type_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>room_type_name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>COMPUTER_LAB</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Компьютерный класс</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>equipment_code</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>equipment_name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>COMPUTERS</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Компьютеры</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="b">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: localize Excel headers to Russian
Makes Russian column labels canonical across all 11 worksheets while retaining complete compatibility with legacy English technical headers.
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R6bd663c9ee7f46dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="R5144b9753eef4871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R0033eb10e51444f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="Raa6879a5fa6047ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Rae5d6d3d1ce345ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R0e5f4c5af9ed4faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R145fb25f3ee6429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="Rbc87389d1d844a5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R68881d1edce44e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R429f29000edb401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="R2d4448ca7fc54ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Raff555a437f64c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rd49f67556cad49ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Rfbc810744b964504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R893de2413b854c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Red4215b796284609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R5e35b220f2094a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R5d13bc032849452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="Re24e0adf775c466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R90b4754672e04171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R8bcaee393170459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="Re70ae7204a114b79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -319,48 +319,48 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="23.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>teacher_code</x:v>
+        <x:v>Код преподавателя</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>full_name</x:v>
+        <x:v>ФИО</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>department</x:v>
+        <x:v>Подразделение</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>employment_type</x:v>
+        <x:v>Тип занятости</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>yearly_assigned_hours</x:v>
+        <x:v>Назначено часов в год</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>yearly_limit_hours</x:v>
+        <x:v>Лимит часов в год</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>max_hours_per_day</x:v>
+        <x:v>Макс. часов в день</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>max_days_per_week</x:v>
+        <x:v>Макс. дней в неделю</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>home_building_code</x:v>
+        <x:v>Основной корпус</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активен</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -405,36 +405,36 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="7.110000133514404" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>room_code</x:v>
+        <x:v>Код аудитории</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>room_name</x:v>
+        <x:v>Название аудитории</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>building_code</x:v>
+        <x:v>Код корпуса</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>room_type_code</x:v>
+        <x:v>Код типа помещения</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>capacity</x:v>
+        <x:v>Вместимость</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>equipment_codes</x:v>
+        <x:v>Коды оборудования</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активна</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -469,76 +469,76 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="21.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="7.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="5.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="17.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="17.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="9" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="16.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="21.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="5.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="21.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>workload_row_code</x:v>
+        <x:v>Код строки нагрузки</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>academic_year</x:v>
+        <x:v>Учебный год</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>semester</x:v>
+        <x:v>Семестр</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>discipline_code</x:v>
+        <x:v>Код дисциплины</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>discipline_name</x:v>
+        <x:v>Название дисциплины</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>group_code</x:v>
+        <x:v>Код группы</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>subgroup</x:v>
+        <x:v>Подгруппа</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>stream</x:v>
+        <x:v>Поток</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>teacher_code</x:v>
+        <x:v>Код преподавателя</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
-        <x:v>lesson_type</x:v>
+        <x:v>Вид занятия</x:v>
       </x:c>
       <x:c r="K1" s="6" t="str">
-        <x:v>total_academic_hours</x:v>
+        <x:v>Всего академических часов</x:v>
       </x:c>
       <x:c r="L1" s="6" t="str">
-        <x:v>event_duration_hours</x:v>
+        <x:v>Продолжительность занятия</x:v>
       </x:c>
       <x:c r="M1" s="6" t="str">
-        <x:v>recurrence</x:v>
+        <x:v>Периодичность</x:v>
       </x:c>
       <x:c r="N1" s="6" t="str">
-        <x:v>lesson_bundle_code</x:v>
+        <x:v>Код связки занятий</x:v>
       </x:c>
       <x:c r="O1" s="6" t="str">
-        <x:v>room_type</x:v>
+        <x:v>Тип помещения</x:v>
       </x:c>
       <x:c r="P1" s="6" t="str">
-        <x:v>room_capacity</x:v>
+        <x:v>Требуемая вместимость</x:v>
       </x:c>
       <x:c r="Q1" s="6" t="str">
-        <x:v>required_equipment_codes</x:v>
+        <x:v>Требуемое оборудование</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -597,48 +597,48 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.889999866485596" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18.110000610351562" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>group_code</x:v>
+        <x:v>Код группы</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>specialty_code</x:v>
+        <x:v>Код специальности</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>curriculum_code</x:v>
+        <x:v>Код учебного плана</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>course</x:v>
+        <x:v>Курс</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>education_form</x:v>
+        <x:v>Форма обучения</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>headcount</x:v>
+        <x:v>Численность</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>program_base</x:v>
+        <x:v>База обучения</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>study_week_type</x:v>
+        <x:v>Тип учебной недели</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>primary_building_code</x:v>
+        <x:v>Основной корпус</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
-        <x:v>subgroup_count</x:v>
+        <x:v>Количество подгрупп</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -682,32 +682,32 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="38.11000061035156" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34.11000061035156" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>specialty_code</x:v>
+        <x:v>Код специальности</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>specialty_name</x:v>
+        <x:v>Название специальности</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>qualification</x:v>
+        <x:v>Квалификация</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>program_base</x:v>
+        <x:v>База обучения</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>education_form</x:v>
+        <x:v>Форма обучения</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активна</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -739,36 +739,36 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="6.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="6.559999942779541" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="5.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.110000133514404" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>curriculum_code</x:v>
+        <x:v>Код учебного плана</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>specialty_code</x:v>
+        <x:v>Код специальности</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>admission_year</x:v>
+        <x:v>Год набора</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>version</x:v>
+        <x:v>Версия</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>valid_from</x:v>
+        <x:v>Действует с</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>valid_to</x:v>
+        <x:v>Действует по</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>status</x:v>
+        <x:v>Статус</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -801,40 +801,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14.220000267028809" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>curriculum_code</x:v>
+        <x:v>Код учебного плана</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>discipline_code</x:v>
+        <x:v>Код дисциплины</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>discipline_name</x:v>
+        <x:v>Название дисциплины</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>section_code</x:v>
+        <x:v>Код раздела</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>semester</x:v>
+        <x:v>Семестр</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>lesson_type</x:v>
+        <x:v>Вид занятия</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>planned_hours</x:v>
+        <x:v>Плановые часы</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>control_form</x:v>
+        <x:v>Форма контроля</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -872,40 +872,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13.890000343322754" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>student_code</x:v>
+        <x:v>Код студента</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>full_name</x:v>
+        <x:v>ФИО</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>group_code</x:v>
+        <x:v>Код группы</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>status</x:v>
+        <x:v>Статус</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>enrollment_date</x:v>
+        <x:v>Дата зачисления</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>end_date</x:v>
+        <x:v>Дата окончания</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>subgroup_codes</x:v>
+        <x:v>Номера подгрупп</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>elective_codes</x:v>
+        <x:v>Коды элективов</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -941,20 +941,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>building_code</x:v>
+        <x:v>Код корпуса</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>building_name</x:v>
+        <x:v>Название корпуса</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активен</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -977,20 +977,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="17.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>room_type_code</x:v>
+        <x:v>Код типа помещения</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>room_type_name</x:v>
+        <x:v>Название типа помещения</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активен</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1013,20 +1013,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="5.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.21999979019165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>equipment_code</x:v>
+        <x:v>Код оборудования</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>equipment_name</x:v>
+        <x:v>Название оборудования</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>active</x:v>
+        <x:v>Активно</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>

<commit_message>
feat: import academic calendar from Excel
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,17 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Raff555a437f64c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rd49f67556cad49ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Rfbc810744b964504"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R893de2413b854c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Red4215b796284609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R5e35b220f2094a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R5d13bc032849452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="Re24e0adf775c466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R90b4754672e04171"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R8bcaee393170459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="Re70ae7204a114b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Re990ba98b8ad466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rd914c15b35df40d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Red8e53b7fac34cf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R7d3bd190be6d40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Rbce6c3d244a6450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R2b5dcc94865d4a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R469519ddbdc4409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="R35a601aa9345426b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R9b1cc6811ca746a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R5fac137cac0042fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="Rfc66e181245143bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные годы" sheetId="12" r:id="Rca02ca4d59594c9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Периоды" sheetId="13" r:id="Rc4471b17980147c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сетка звонков" sheetId="14" r:id="Rd8846b9bb286499c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -593,6 +596,170 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.21999979019165" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Дата начала</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Дата окончания</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Активен</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="n">
+        <x:v>46568</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="7.559999942779541" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Код периода</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Название периода</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Тип периода</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Дата начала</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Дата окончания</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>Семестр</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>SEM-1</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Первый семестр</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>teaching</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="n">
+        <x:v>46384</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="6.440000057220459" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.4399995803833" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Код интервала</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Код смены</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Номер занятия</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Начало</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Окончание</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>S1-01</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>S1</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>08:30</x:v>
+      </x:c>
+      <x:c r="F2" s="7" t="str">
+        <x:v>10:00</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
feat: import calendar constraints from Excel
Add holidays, shortened and transferred days plus resource unavailability as an optional two-sheet calendar extension. Persist the new records atomically, expose their counts in CLI and web previews, and keep legacy 14-sheet calendar files compatible.
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,20 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="Re990ba98b8ad466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rd914c15b35df40d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="Red8e53b7fac34cf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R7d3bd190be6d40dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="Rbce6c3d244a6450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="R2b5dcc94865d4a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R469519ddbdc4409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="R35a601aa9345426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="R9b1cc6811ca746a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R5fac137cac0042fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="Rfc66e181245143bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные годы" sheetId="12" r:id="Rca02ca4d59594c9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Периоды" sheetId="13" r:id="Rc4471b17980147c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сетка звонков" sheetId="14" r:id="Rd8846b9bb286499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R6364164231f54b1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rc78341c64dec4a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R06c3de5521c543a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R942ab6487ebf42e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R5cbb9b859a5240b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="Ra5a0bdeb17854d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R9b5dcb8ddd9e4dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="R90f14cd59cbc40f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="Rac2062f696b04f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R601445eb8e31472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="R4042dc217eb6478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные годы" sheetId="12" r:id="Rb1ae75a38b2e4027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Периоды" sheetId="13" r:id="R9d63dd377f8b4df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сетка звонков" sheetId="14" r:id="Ra39f26d6bbce4373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исключения календаря" sheetId="15" r:id="R63ad4b258f2d4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Недоступность" sheetId="16" r:id="R0d932fcb491b4ee9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -760,6 +762,140 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20.440000534057617" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Код исключения</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Тип исключения</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Дата исключения</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Перенос на дату</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Сокращённый день до</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>Примечание</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>EX-001</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>holiday</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="n">
+        <x:v>46330</x:v>
+      </x:c>
+      <x:c r="E2" s="9"/>
+      <x:c r="F2" s="7"/>
+      <x:c r="G2" s="7" t="str">
+        <x:v>День народного единства</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="21.110000610351562" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Код недоступности</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Тип ресурса</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Код ресурса</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Дата начала</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Дата окончания</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>Время начала</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>Время окончания</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>Причина</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>U-001</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>teacher</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>T-001</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>46296</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
+      <x:c r="I2" s="7" t="str">
+        <x:v>Повышение квалификации</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
feat: support academic week cycles
</commit_message>
<xml_diff>
--- a/tests/fixtures/formula-import.xlsx
+++ b/tests/fixtures/formula-import.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R6364164231f54b1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rc78341c64dec4a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R06c3de5521c543a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R942ab6487ebf42e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R5cbb9b859a5240b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="Ra5a0bdeb17854d95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R9b5dcb8ddd9e4dd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="R90f14cd59cbc40f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="Rac2062f696b04f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="R601445eb8e31472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="R4042dc217eb6478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные годы" sheetId="12" r:id="Rb1ae75a38b2e4027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Периоды" sheetId="13" r:id="R9d63dd377f8b4df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сетка звонков" sheetId="14" r:id="Ra39f26d6bbce4373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исключения календаря" sheetId="15" r:id="R63ad4b258f2d4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Недоступность" sheetId="16" r:id="R0d932fcb491b4ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Преподаватели" sheetId="1" r:id="R1dd9334854fc4e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="2" r:id="Rdbf701a024c34ef1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Специальности" sheetId="3" r:id="R04e293caff5f4698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные планы" sheetId="4" r:id="R3749ec94a9f2460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дисциплины" sheetId="5" r:id="R411d645f05d442ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Студенты" sheetId="6" r:id="Rbd7256ee2e7642c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Корпуса" sheetId="7" r:id="R830c6b568a61488f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Типы помещений" sheetId="8" r:id="R9a45b17bf88441bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оборудование" sheetId="9" r:id="Rec1c9181288c45cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудитории" sheetId="10" r:id="Rfd17f49251b0401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузка" sheetId="11" r:id="R13a559467adf4700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные годы" sheetId="12" r:id="R9d6316d0e84549ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Учебные циклы" sheetId="13" r:id="Rad8cfccc6b2e4d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Периоды" sheetId="14" r:id="R2b0273a47301467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сетка звонков" sheetId="15" r:id="R5f3eb102a767443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исключения календаря" sheetId="16" r:id="R70948f89131245bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Недоступность" sheetId="17" r:id="R36e74876b92046e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -491,6 +492,8 @@
     <x:col min="15" max="15" width="13.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="20.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="21.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="23" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18.219999313354492" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -544,6 +547,12 @@
       </x:c>
       <x:c r="Q1" s="6" t="str">
         <x:v>Требуемое оборудование</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>Код учебного цикла</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>Номера недель цикла</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -592,6 +601,12 @@
       <x:c r="Q2" s="7" t="str">
         <x:v>COMPUTERS</x:v>
       </x:c>
+      <x:c r="R2" s="7" t="str">
+        <x:v>NUMERATOR-DENOMINATOR</x:v>
+      </x:c>
+      <x:c r="S2" s="7" t="str">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -642,6 +657,63 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.21999979019165" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>Код цикла</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>Учебный год</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>Название цикла</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Длина цикла в неделях</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>Дата начала отсчёта</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Активен</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>NUMERATOR-DENOMINATOR</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026/2027</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>Числитель / знаменатель</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -705,7 +777,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -762,7 +834,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -822,7 +894,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>

</xml_diff>